<commit_message>
updated selenium and appium automation on Feb 7th 2021
</commit_message>
<xml_diff>
--- a/testdata/TestData.xlsx
+++ b/testdata/TestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11014"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookpro/eclipse-workspace/XOME/testdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/geeky/OneDrive/eclipse-workspace/XOME/testdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CACB38D-6AFE-3E4E-9E63-87FEEDCA52E5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{2CACB38D-6AFE-3E4E-9E63-87FEEDCA52E5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{E3718968-7744-9548-AEB9-9967C4967813}"/>
   <bookViews>
-    <workbookView xWindow="820" yWindow="9880" windowWidth="27980" windowHeight="7320" activeTab="3" xr2:uid="{9E591401-0C67-8242-A747-6951EB72A76F}"/>
+    <workbookView xWindow="820" yWindow="9880" windowWidth="27980" windowHeight="7320" activeTab="7" xr2:uid="{9E591401-0C67-8242-A747-6951EB72A76F}"/>
   </bookViews>
   <sheets>
     <sheet name="signUpWithBlankFields" sheetId="1" r:id="rId1"/>
@@ -158,10 +158,10 @@
     <t>TESTER</t>
   </si>
   <si>
-    <t>12512 Brighton Place Tustin, CA 92780</t>
-  </si>
-  <si>
     <t>wontshare</t>
+  </si>
+  <si>
+    <t>12512 Brighton Pl Tustin, CA 92780</t>
   </si>
 </sst>
 </file>
@@ -1115,7 +1115,7 @@
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
         <v>14</v>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="2" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>